<commit_message>
don't user normalize-space which enketo supported but not mobile
</commit_message>
<xml_diff>
--- a/iaso/tests/fixtures/form_with_org_unit_groups_injectables.xlsx
+++ b/iaso/tests/fixtures/form_with_org_unit_groups_injectables.xlsx
@@ -621,7 +621,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>normalize-space(concat(${current_ou_group_ids}, ' ', ${parent1_ou_group_ids}, ' ', ${parent2_ou_group_ids}))</t>
+          <t>concat(${current_ou_group_ids}, ' ', ${parent1_ou_group_ids}, ' ', ${parent2_ou_group_ids})</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>normalize-space(concat(${current_ou_group_names}, ' ', ${parent1_ou_group_names}, ' ', ${parent2_ou_group_names}))</t>
+          <t>concat(${current_ou_group_names}, ' ', ${parent1_ou_group_names}, ' ', ${parent2_ou_group_names})</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>if(selected(${all_group_ids}, string(${group_id_to_check})), 1, 0)</t>
+          <t>if(${group_id_to_check} != '' and selected(${all_group_ids}, string(${group_id_to_check})), 1, 0)</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026100803</t>
+          <t>2026101301</t>
         </is>
       </c>
     </row>

</xml_diff>